<commit_message>
Formatea la hoja vitrina como planilla de pastelería
La plantilla deja de ser un CSV crudo: títulos en español, menú si/no,
notas de producto y una pestaña Cómo usar. La página ya entiende esos encabezados.

Co-authored-by: simpleideal <simpleideal@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/demo-vitrina/datos/plantilla-google-sheets.xlsx
+++ b/demo-vitrina/datos/plantilla-google-sheets.xlsx
@@ -7,11 +7,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="ofertas" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="como_usar" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Hoja 1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Cómo usar" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ofertas'!$A$1:$I$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Hoja 1'!$A$1:$I$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -40,7 +40,7 @@
       <sz val="14"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -60,6 +60,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF7E3C6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF4D4C8"/>
       </patternFill>
     </fill>
   </fills>
@@ -89,7 +94,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -100,10 +105,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -195,64 +203,64 @@
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
         <t>Nombre que ve el cliente. No lo dejes vacío.
-No cambies estos nombres.
-Esta pestaña tiene que llamarse ofertas.</t>
+No cambies estos títulos.
+La vitrina lee esta pestaña.</t>
       </text>
     </comment>
     <comment ref="B1" authorId="0" shapeId="0">
       <text>
         <t>Precio de vitrina, solo números, sin $.
-No cambies estos nombres.
-Esta pestaña tiene que llamarse ofertas.</t>
+No cambies estos títulos.
+La vitrina lee esta pestaña.</t>
       </text>
     </comment>
     <comment ref="C1" authorId="0" shapeId="0">
       <text>
         <t>Precio de hoy. Si va vacío, se usa el normal.
-No cambies estos nombres.
-Esta pestaña tiene que llamarse ofertas.</t>
+No cambies estos títulos.
+La vitrina lee esta pestaña.</t>
       </text>
     </comment>
     <comment ref="D1" authorId="0" shapeId="0">
       <text>
         <t>si o no. Solo si sale en la vitrina.
-No cambies estos nombres.
-Esta pestaña tiene que llamarse ofertas.</t>
+No cambies estos títulos.
+La vitrina lee esta pestaña.</t>
       </text>
     </comment>
     <comment ref="E1" authorId="0" shapeId="0">
       <text>
         <t>si o no. no = ni se publica.
-No cambies estos nombres.
-Esta pestaña tiene que llamarse ofertas.</t>
+No cambies estos títulos.
+La vitrina lee esta pestaña.</t>
       </text>
     </comment>
     <comment ref="F1" authorId="0" shapeId="0">
       <text>
         <t>Una línea. Puede ir vacía.
-No cambies estos nombres.
-Esta pestaña tiene que llamarse ofertas.</t>
+No cambies estos títulos.
+La vitrina lee esta pestaña.</t>
       </text>
     </comment>
     <comment ref="G1" authorId="0" shapeId="0">
       <text>
-        <t>URL https://… o vacío. En Drive: cualquiera con el enlace.
-No cambies estos nombres.
-Esta pestaña tiene que llamarse ofertas.</t>
+        <t>URL https://… o vacío.
+No cambies estos títulos.
+La vitrina lee esta pestaña.</t>
       </text>
     </comment>
     <comment ref="H1" authorId="0" shapeId="0">
       <text>
         <t>Número. 0 = Agotado. Vacío = no se muestra el cupo.
-No cambies estos nombres.
-Esta pestaña tiene que llamarse ofertas.</t>
+No cambies estos títulos.
+La vitrina lee esta pestaña.</t>
       </text>
     </comment>
     <comment ref="I1" authorId="0" shapeId="0">
       <text>
         <t>Opcional. Agrupa: Horno, Para llevar…
-No cambies estos nombres.
-Esta pestaña tiene que llamarse ofertas.</t>
+No cambies estos títulos.
+La vitrina lee esta pestaña.</t>
       </text>
     </comment>
   </commentList>
@@ -566,47 +574,47 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>producto</t>
+          <t>Producto</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>precio_normal</t>
+          <t>Precio normal</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>precio_oferta</t>
+          <t>Precio oferta</t>
         </is>
       </c>
       <c r="D1" s="2" t="inlineStr">
         <is>
-          <t>hoy</t>
+          <t>Hoy</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>activo</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>nota</t>
+          <t>Nota</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>foto</t>
+          <t>Foto</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>unidades</t>
+          <t>Unidades</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>categoria</t>
+          <t>Categoría</t>
         </is>
       </c>
     </row>
@@ -634,7 +642,7 @@
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>Márcalo si para liquidar hoy. La foto es opcional.</t>
+          <t>Queda de la mañana</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr"/>
@@ -659,7 +667,7 @@
       <c r="C3" s="4" t="n">
         <v>3900</v>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -671,7 +679,7 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Activo pero hoy=no: no sale en la vitrina.</t>
+          <t>Sale mañana fresco</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr"/>
@@ -708,7 +716,7 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Unidades vacío: se muestra sin cupo.</t>
+          <t>Pack para llevar</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr"/>
@@ -743,11 +751,11 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>unidades=0 se ve Agotado.</t>
+          <t>Se acabó</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr"/>
-      <c r="H5" s="4" t="n">
+      <c r="H5" s="6" t="n">
         <v>0</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
@@ -768,7 +776,7 @@
       <c r="C6" s="4" t="n">
         <v>24900</v>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -780,7 +788,7 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>activo=no: el cliente no lo ve nunca.</t>
+          <t>Solo por encargo</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr"/>
@@ -796,7 +804,7 @@
   </sheetData>
   <autoFilter ref="A1:I6"/>
   <dataValidations count="1">
-    <dataValidation sqref="D2:D200 E2:E200" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Usa si o no" error="Escribe si o no, en minúscula." promptTitle="Hoy / activo" prompt="si o no" type="list">
+    <dataValidation sqref="D2:D200 E2:E200" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Usa si o no" error="Elige si o no, en minúscula." promptTitle="Hoy / Activo" prompt="si o no" type="list">
       <formula1>"si,no"</formula1>
     </dataValidation>
   </dataValidations>
@@ -812,122 +820,112 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A19"/>
+  <dimension ref="A1:A17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="88" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>Cómo usar esta hoja (el local no entra a GitHub)</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
-      <c r="A2" s="7" t="inlineStr"/>
+      <c r="A2" s="8" t="inlineStr"/>
     </row>
     <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="7" t="inlineStr">
-        <is>
-          <t>Esta pestaña no se publica. La vitrina lee solo la pestaña ofertas.</t>
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>Esta pestaña no se publica. La vitrina lee solo Hoja 1.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="7" t="inlineStr"/>
+      <c r="A4" s="8" t="inlineStr"/>
     </row>
     <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>Cada tarde:</t>
         </is>
       </c>
     </row>
     <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="7" t="inlineStr">
-        <is>
-          <t>1. En lo que quieres liquidar: hoy = si. Completa precio_oferta y unidades.</t>
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>1. Lo que quieres liquidar: Hoy = si. Completa Precio oferta y Unidades.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>2. En lo demás: hoy = no.</t>
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>2. Lo demás: Hoy = no.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1">
-      <c r="A8" s="7" t="inlineStr">
-        <is>
-          <t>3. Si se acabó: unidades = 0 (sale Agotado).</t>
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>3. Si se acabó: Unidades = 0 (sale Agotado).</t>
         </is>
       </c>
     </row>
     <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="7" t="inlineStr">
-        <is>
-          <t>4. Si un producto no debe verse nunca: activo = no.</t>
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>4. Si un producto no debe verse nunca: Activo = no.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="7" t="inlineStr"/>
+      <c r="A10" s="8" t="inlineStr"/>
     </row>
     <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="7" t="inlineStr">
-        <is>
-          <t>No cambies la fila 1 ni el nombre de la pestaña ofertas.</t>
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>No cambies la fila 1 (los títulos verdes).</t>
         </is>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="7" t="inlineStr">
+      <c r="A12" s="8" t="inlineStr">
         <is>
           <t>No pongas $ en los precios. Solo el número: 4500.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="7" t="inlineStr">
-        <is>
-          <t>foto puede ir vacía. Si pegas un enlace de Drive, que sea “cualquiera con el enlace”.</t>
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>Foto puede ir vacía.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="7" t="inlineStr"/>
+      <c r="A14" s="8" t="inlineStr"/>
     </row>
     <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="7" t="inlineStr">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>Hoy y Activo tienen un menú: elige si o no.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" s="8" t="inlineStr">
         <is>
           <t>Una vez (Simple Ideal): Compartir → cualquiera con el enlace puede ver.</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="18" customHeight="1">
-      <c r="A16" s="7" t="inlineStr">
-        <is>
-          <t>Copia el enlace de la hoja y pégalo en DATOS DE LA VITRINA → hoja.</t>
-        </is>
-      </c>
-    </row>
     <row r="17" ht="18" customHeight="1">
-      <c r="A17" s="7" t="inlineStr">
-        <is>
-          <t>El llavero NFC y el QR siguen abriendo la misma URL.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="18" customHeight="1">
-      <c r="A18" s="7" t="inlineStr"/>
-    </row>
-    <row r="19" ht="18" customHeight="1">
-      <c r="A19" s="7" t="inlineStr">
-        <is>
-          <t>Para otro local: Archivo → Hacer una copia. Cada pastelería tiene su hoja.</t>
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>Para otro local: Archivo → Hacer una copia.</t>
         </is>
       </c>
     </row>

</xml_diff>